<commit_message>
add pruned vals manually
</commit_message>
<xml_diff>
--- a/metrics/Example.xlsx
+++ b/metrics/Example.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="22">
   <si>
     <t>Validator Address</t>
   </si>
@@ -81,20 +81,26 @@
     <t>Uptime</t>
   </si>
   <si>
-    <t>Overall</t>
-  </si>
-  <si>
     <t>Blocks Range &gt;&gt;&gt;</t>
   </si>
   <si>
-    <t>https://stackoverflow.com/questions/37434227/how-to-open-xlsx-file-with-python-3</t>
+    <t>Total Signed #</t>
+  </si>
+  <si>
+    <t>Total Missed #</t>
+  </si>
+  <si>
+    <t>Avg Uptime per day</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="9" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="0.000%"/>
+  </numFmts>
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -151,13 +157,6 @@
       <charset val="204"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="204"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color theme="10"/>
@@ -166,8 +165,23 @@
       <charset val="204"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0" tint="-0.34998626667073579"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0" tint="-0.34998626667073579"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -198,8 +212,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="16">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -260,17 +280,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -320,46 +329,7 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
+      <right/>
       <top/>
       <bottom/>
       <diagonal/>
@@ -369,9 +339,16 @@
         <color indexed="64"/>
       </left>
       <right/>
-      <top style="thin">
+      <top/>
+      <bottom style="medium">
         <color indexed="64"/>
-      </top>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -382,9 +359,7 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
+      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -393,9 +368,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -404,92 +379,18 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="2" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="2" fillId="5" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -498,13 +399,102 @@
     <xf numFmtId="14" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="2" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
@@ -538,6 +528,7 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1092,6 +1083,7 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1990,6 +1982,7 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -4529,22 +4522,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
     <col min="2" max="2" width="56.77734375" customWidth="1"/>
     <col min="3" max="3" width="16.6640625" customWidth="1"/>
-    <col min="4" max="5" width="17.6640625" customWidth="1"/>
-    <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.33203125" customWidth="1"/>
-    <col min="8" max="8" width="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="17.6640625" customWidth="1"/>
+    <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.33203125" customWidth="1"/>
+    <col min="11" max="11" width="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
@@ -4558,409 +4552,485 @@
         <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1" s="10">
+        <v>45590</v>
+      </c>
+      <c r="J1" s="24"/>
+      <c r="K1" s="10">
+        <v>45591</v>
+      </c>
+      <c r="L1" s="24"/>
+      <c r="M1" s="10">
+        <v>45592</v>
+      </c>
+      <c r="N1" s="11"/>
+    </row>
+    <row r="2" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="34">
-        <v>45590</v>
-      </c>
-      <c r="G1" s="35"/>
-      <c r="H1" s="34">
-        <v>45591</v>
-      </c>
-      <c r="I1" s="35"/>
-      <c r="J1" s="34">
-        <v>45592</v>
-      </c>
-      <c r="K1" s="35"/>
-    </row>
-    <row r="2" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="16" t="s">
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="17"/>
-      <c r="H2" s="16" t="s">
+      <c r="J2" s="32"/>
+      <c r="K2" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="I2" s="17"/>
-      <c r="J2" s="16" t="s">
+      <c r="L2" s="32"/>
+      <c r="M2" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="K2" s="17"/>
-    </row>
-    <row r="3" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="18" t="s">
+      <c r="N2" s="33"/>
+    </row>
+    <row r="3" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="24">
+      <c r="D3" s="7">
         <v>1</v>
       </c>
-      <c r="E3" s="10">
-        <f>SUM(F5:K5)/COUNT(F5:K5)</f>
+      <c r="E3" s="7">
+        <v>458944</v>
+      </c>
+      <c r="F3" s="7">
+        <v>798</v>
+      </c>
+      <c r="G3" s="34">
+        <f>E3/(E3+F3)</f>
+        <v>0.99826424385851198</v>
+      </c>
+      <c r="H3" s="37">
+        <f>SUM(I5:N5)/COUNT(I5:N5)</f>
         <v>0.96085447712521399</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="I3" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="J3" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="K3" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="L3" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="M3" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="N3" s="39" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="19"/>
-      <c r="B4" s="21"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="6">
+    <row r="4" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="18"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="38"/>
+      <c r="I4" s="26">
         <v>837</v>
       </c>
-      <c r="G4" s="7">
+      <c r="J4" s="23">
         <v>32</v>
       </c>
-      <c r="H4" s="6">
+      <c r="K4" s="26">
         <v>814</v>
       </c>
-      <c r="I4" s="7">
+      <c r="L4" s="23">
         <v>12</v>
       </c>
-      <c r="J4" s="6">
+      <c r="M4" s="26">
         <v>749</v>
       </c>
-      <c r="K4" s="7">
+      <c r="N4" s="4">
         <v>53</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="19"/>
-      <c r="B5" s="21"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="36">
-        <f>F4/(F4+G4)</f>
+    <row r="5" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="18"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="36"/>
+      <c r="H5" s="40"/>
+      <c r="I5" s="41">
+        <f>I4/(I4+J4)</f>
         <v>0.96317606444188719</v>
       </c>
-      <c r="G5" s="37"/>
-      <c r="H5" s="36">
-        <f>H4/(H4+I4)</f>
+      <c r="J5" s="42"/>
+      <c r="K5" s="41">
+        <f>K4/(K4+L4)</f>
         <v>0.98547215496368035</v>
       </c>
-      <c r="I5" s="37"/>
-      <c r="J5" s="36">
-        <f>J4/(J4+K4)</f>
+      <c r="L5" s="42"/>
+      <c r="M5" s="41">
+        <f>M4/(M4+N4)</f>
         <v>0.93391521197007477</v>
       </c>
-      <c r="K5" s="37"/>
-    </row>
-    <row r="6" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="18" t="s">
+      <c r="N5" s="43"/>
+    </row>
+    <row r="6" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="24">
-        <v>0</v>
-      </c>
-      <c r="E6" s="10">
-        <f t="shared" ref="E6" si="0">SUM(F8:K8)/COUNT(F8:K8)</f>
-        <v>0.97804012478974922</v>
-      </c>
-      <c r="F6" s="4" t="s">
+      <c r="D6" s="7">
+        <v>0</v>
+      </c>
+      <c r="E6" s="7">
+        <v>408735</v>
+      </c>
+      <c r="F6" s="7">
+        <v>12765</v>
+      </c>
+      <c r="G6" s="34">
+        <f t="shared" ref="G6" si="0">E6/(E6+F6)</f>
+        <v>0.96971530249110316</v>
+      </c>
+      <c r="H6" s="37">
+        <f>SUM(I8:N8)/COUNT(I8:N8)</f>
+        <v>0.97580162357069866</v>
+      </c>
+      <c r="I6" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="J6" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="K6" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="L6" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="M6" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="N6" s="39" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="19"/>
-      <c r="B7" s="21"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="6">
+    <row r="7" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="18"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="35"/>
+      <c r="H7" s="38"/>
+      <c r="I7" s="26">
         <v>837</v>
       </c>
-      <c r="G7" s="8">
+      <c r="J7" s="23">
+        <v>42</v>
+      </c>
+      <c r="K7" s="26">
+        <v>814</v>
+      </c>
+      <c r="L7" s="23">
+        <v>12</v>
+      </c>
+      <c r="M7" s="26">
+        <v>866</v>
+      </c>
+      <c r="N7" s="4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="18"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="36"/>
+      <c r="H8" s="40"/>
+      <c r="I8" s="41">
+        <f>I7/(I7+J7)</f>
+        <v>0.95221843003412965</v>
+      </c>
+      <c r="J8" s="42"/>
+      <c r="K8" s="41">
+        <f>K7/(K7+L7)</f>
+        <v>0.98547215496368035</v>
+      </c>
+      <c r="L8" s="42"/>
+      <c r="M8" s="41">
+        <f>M7/(M7+N7)</f>
+        <v>0.98971428571428577</v>
+      </c>
+      <c r="N8" s="43"/>
+    </row>
+    <row r="9" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="7">
+        <v>1</v>
+      </c>
+      <c r="E9" s="7">
+        <v>858934</v>
+      </c>
+      <c r="F9" s="7">
+        <v>2893</v>
+      </c>
+      <c r="G9" s="34">
+        <f t="shared" ref="G9" si="1">E9/(E9+F9)</f>
+        <v>0.99664317780714695</v>
+      </c>
+      <c r="H9" s="37">
+        <f t="shared" ref="H9" si="2">SUM(I11:N11)/COUNT(I11:N11)</f>
+        <v>0.95498767758068537</v>
+      </c>
+      <c r="I9" s="27" t="s">
+        <v>2</v>
+      </c>
+      <c r="J9" s="25" t="s">
+        <v>3</v>
+      </c>
+      <c r="K9" s="27" t="s">
+        <v>2</v>
+      </c>
+      <c r="L9" s="25" t="s">
+        <v>3</v>
+      </c>
+      <c r="M9" s="27" t="s">
+        <v>2</v>
+      </c>
+      <c r="N9" s="39" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="18"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="35"/>
+      <c r="H10" s="38"/>
+      <c r="I10" s="26">
+        <v>837</v>
+      </c>
+      <c r="J10" s="23">
+        <v>13</v>
+      </c>
+      <c r="K10" s="26">
+        <v>814</v>
+      </c>
+      <c r="L10" s="23">
+        <v>12</v>
+      </c>
+      <c r="M10" s="26">
+        <v>978</v>
+      </c>
+      <c r="N10" s="4">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="18"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="36"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="41">
+        <f>I10/(I10+J10)</f>
+        <v>0.98470588235294121</v>
+      </c>
+      <c r="J11" s="42"/>
+      <c r="K11" s="41">
+        <f>K10/(K10+L10)</f>
+        <v>0.98547215496368035</v>
+      </c>
+      <c r="L11" s="42"/>
+      <c r="M11" s="41">
+        <f>M10/(M10+N10)</f>
+        <v>0.89478499542543455</v>
+      </c>
+      <c r="N11" s="43"/>
+    </row>
+    <row r="12" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="7">
+        <v>2</v>
+      </c>
+      <c r="E12" s="7">
+        <v>148718</v>
+      </c>
+      <c r="F12" s="7">
+        <v>189</v>
+      </c>
+      <c r="G12" s="34">
+        <f t="shared" ref="G12" si="3">E12/(E12+F12)</f>
+        <v>0.99873075140859735</v>
+      </c>
+      <c r="H12" s="37">
+        <f t="shared" ref="H12" si="4">SUM(I14:N14)/COUNT(I14:N14)</f>
+        <v>0.9568351746829431</v>
+      </c>
+      <c r="I12" s="27" t="s">
+        <v>2</v>
+      </c>
+      <c r="J12" s="25" t="s">
+        <v>3</v>
+      </c>
+      <c r="K12" s="27" t="s">
+        <v>2</v>
+      </c>
+      <c r="L12" s="25" t="s">
+        <v>3</v>
+      </c>
+      <c r="M12" s="27" t="s">
+        <v>2</v>
+      </c>
+      <c r="N12" s="39" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="18"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="35"/>
+      <c r="H13" s="38"/>
+      <c r="I13" s="26">
+        <v>837</v>
+      </c>
+      <c r="J13" s="23">
         <v>32</v>
       </c>
-      <c r="H7" s="6">
+      <c r="K13" s="26">
         <v>814</v>
       </c>
-      <c r="I7" s="8">
+      <c r="L13" s="23">
+        <v>69</v>
+      </c>
+      <c r="M13" s="26">
+        <v>814</v>
+      </c>
+      <c r="N13" s="4">
         <v>12</v>
       </c>
-      <c r="J7" s="6">
-        <v>814</v>
-      </c>
-      <c r="K7" s="8">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="19"/>
-      <c r="B8" s="21"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="36">
-        <f>F7/(F7+G7)</f>
+    </row>
+    <row r="14" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="19"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="36"/>
+      <c r="H14" s="40"/>
+      <c r="I14" s="41">
+        <f>I13/(I13+J13)</f>
         <v>0.96317606444188719</v>
       </c>
-      <c r="G8" s="37"/>
-      <c r="H8" s="36">
-        <f>H7/(H7+I7)</f>
+      <c r="J14" s="42"/>
+      <c r="K14" s="41">
+        <f>K13/(K13+L13)</f>
+        <v>0.92185730464326165</v>
+      </c>
+      <c r="L14" s="42"/>
+      <c r="M14" s="41">
+        <f>M13/(M13+N13)</f>
         <v>0.98547215496368035</v>
       </c>
-      <c r="I8" s="37"/>
-      <c r="J8" s="36">
-        <f>J7/(J7+K7)</f>
-        <v>0.98547215496368035</v>
-      </c>
-      <c r="K8" s="37"/>
-    </row>
-    <row r="9" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="C9" s="28" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="24">
-        <v>0</v>
-      </c>
-      <c r="E9" s="10">
-        <f t="shared" ref="E9" si="1">SUM(F11:K11)/COUNT(F11:K11)</f>
-        <v>0.97804012478974922</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K9" s="5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="19"/>
-      <c r="B10" s="21"/>
-      <c r="C10" s="29"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="6">
-        <v>837</v>
-      </c>
-      <c r="G10" s="8">
-        <v>32</v>
-      </c>
-      <c r="H10" s="6">
-        <v>814</v>
-      </c>
-      <c r="I10" s="8">
-        <v>12</v>
-      </c>
-      <c r="J10" s="6">
-        <v>814</v>
-      </c>
-      <c r="K10" s="8">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="19"/>
-      <c r="B11" s="21"/>
-      <c r="C11" s="29"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="36">
-        <f>F10/(F10+G10)</f>
-        <v>0.96317606444188719</v>
-      </c>
-      <c r="G11" s="37"/>
-      <c r="H11" s="36">
-        <f>H10/(H10+I10)</f>
-        <v>0.98547215496368035</v>
-      </c>
-      <c r="I11" s="37"/>
-      <c r="J11" s="36">
-        <f>J10/(J10+K10)</f>
-        <v>0.98547215496368035</v>
-      </c>
-      <c r="K11" s="37"/>
-    </row>
-    <row r="12" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="25" t="s">
-        <v>8</v>
-      </c>
-      <c r="B12" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="C12" s="22" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12" s="24">
-        <v>2</v>
-      </c>
-      <c r="E12" s="10">
-        <f t="shared" ref="E12" si="2">SUM(F14:K14)/COUNT(F14:K14)</f>
-        <v>0.97804012478974922</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="I12" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K12" s="5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="26"/>
-      <c r="B13" s="21"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="6">
-        <v>837</v>
-      </c>
-      <c r="G13" s="8">
-        <v>32</v>
-      </c>
-      <c r="H13" s="6">
-        <v>814</v>
-      </c>
-      <c r="I13" s="8">
-        <v>12</v>
-      </c>
-      <c r="J13" s="6">
-        <v>814</v>
-      </c>
-      <c r="K13" s="8">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="27"/>
-      <c r="B14" s="31"/>
-      <c r="C14" s="30"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="32">
-        <f>F13/(F13+G13)</f>
-        <v>0.96317606444188719</v>
-      </c>
-      <c r="G14" s="33"/>
-      <c r="H14" s="32">
-        <f>H13/(H13+I13)</f>
-        <v>0.98547215496368035</v>
-      </c>
-      <c r="I14" s="33"/>
-      <c r="J14" s="32">
-        <f>J13/(J13+K13)</f>
-        <v>0.98547215496368035</v>
-      </c>
-      <c r="K14" s="33"/>
+      <c r="N14" s="43"/>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B17" s="38" t="s">
-        <v>20</v>
-      </c>
+      <c r="B17" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="39">
-    <mergeCell ref="D9:D11"/>
-    <mergeCell ref="E6:E8"/>
-    <mergeCell ref="E9:E11"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="B12:B14"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="D3:D5"/>
-    <mergeCell ref="D6:D8"/>
-    <mergeCell ref="B6:B8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="B9:B11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="J11:K11"/>
+  <mergeCells count="51">
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="F3:F5"/>
+    <mergeCell ref="F6:F8"/>
+    <mergeCell ref="F9:F11"/>
+    <mergeCell ref="F12:F14"/>
+    <mergeCell ref="G3:G5"/>
+    <mergeCell ref="H3:H5"/>
+    <mergeCell ref="H6:H8"/>
+    <mergeCell ref="H9:H11"/>
+    <mergeCell ref="H12:H14"/>
+    <mergeCell ref="G6:G8"/>
+    <mergeCell ref="G9:G11"/>
+    <mergeCell ref="G12:G14"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="M5:N5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="K14:L14"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="K11:L11"/>
+    <mergeCell ref="M11:N11"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="I8:J8"/>
     <mergeCell ref="E12:E14"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="C3:C5"/>
@@ -4972,12 +5042,19 @@
     <mergeCell ref="C6:C8"/>
     <mergeCell ref="C9:C11"/>
     <mergeCell ref="C12:C14"/>
+    <mergeCell ref="B12:B14"/>
+    <mergeCell ref="D3:D5"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="D9:D11"/>
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="E9:E11"/>
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="I2:J2"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="B17" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -5013,7 +5090,7 @@
       <c r="C2">
         <v>2</v>
       </c>
-      <c r="D2" s="9">
+      <c r="D2" s="5">
         <f>B2/(B2+C2)</f>
         <v>0.98639455782312924</v>
       </c>
@@ -5028,7 +5105,7 @@
       <c r="C3">
         <v>4</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="5">
         <f t="shared" ref="D3:D40" si="0">B3/(B3+C3)</f>
         <v>0.97385620915032678</v>
       </c>
@@ -5043,7 +5120,7 @@
       <c r="C4">
         <v>6</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="5">
         <f t="shared" si="0"/>
         <v>0.96226415094339623</v>
       </c>
@@ -5058,7 +5135,7 @@
       <c r="C5">
         <v>8</v>
       </c>
-      <c r="D5" s="9">
+      <c r="D5" s="5">
         <f t="shared" si="0"/>
         <v>0.95151515151515154</v>
       </c>
@@ -5073,7 +5150,7 @@
       <c r="C6">
         <v>10</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="5">
         <f t="shared" si="0"/>
         <v>0.94152046783625731</v>
       </c>
@@ -5088,7 +5165,7 @@
       <c r="C7">
         <v>12</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="5">
         <f t="shared" si="0"/>
         <v>0.93220338983050843</v>
       </c>
@@ -5103,7 +5180,7 @@
       <c r="C8">
         <v>14</v>
       </c>
-      <c r="D8" s="9">
+      <c r="D8" s="5">
         <f t="shared" si="0"/>
         <v>0.92349726775956287</v>
       </c>
@@ -5118,7 +5195,7 @@
       <c r="C9">
         <v>16</v>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="5">
         <f t="shared" si="0"/>
         <v>0.91534391534391535</v>
       </c>
@@ -5133,7 +5210,7 @@
       <c r="C10">
         <v>18</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="5">
         <f t="shared" si="0"/>
         <v>0.90769230769230769</v>
       </c>
@@ -5142,7 +5219,7 @@
       <c r="A11" s="1">
         <v>45599</v>
       </c>
-      <c r="D11" s="9"/>
+      <c r="D11" s="5"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
@@ -5154,7 +5231,7 @@
       <c r="C12">
         <v>22</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="5">
         <f t="shared" si="0"/>
         <v>0.893719806763285</v>
       </c>
@@ -5169,7 +5246,7 @@
       <c r="C13">
         <v>24</v>
       </c>
-      <c r="D13" s="9">
+      <c r="D13" s="5">
         <f t="shared" si="0"/>
         <v>0.88732394366197187</v>
       </c>
@@ -5184,7 +5261,7 @@
       <c r="C14">
         <v>3</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="5">
         <f t="shared" si="0"/>
         <v>0.98469387755102045</v>
       </c>
@@ -5199,7 +5276,7 @@
       <c r="C15">
         <v>28</v>
       </c>
-      <c r="D15" s="9">
+      <c r="D15" s="5">
         <f t="shared" si="0"/>
         <v>0.87555555555555553</v>
       </c>
@@ -5214,7 +5291,7 @@
       <c r="C16">
         <v>30</v>
       </c>
-      <c r="D16" s="9">
+      <c r="D16" s="5">
         <f t="shared" si="0"/>
         <v>0.87012987012987009</v>
       </c>
@@ -5229,7 +5306,7 @@
       <c r="C17">
         <v>4</v>
       </c>
-      <c r="D17" s="9">
+      <c r="D17" s="5">
         <f t="shared" si="0"/>
         <v>0.98086124401913877</v>
       </c>
@@ -5244,7 +5321,7 @@
       <c r="C18">
         <v>34</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="5">
         <f t="shared" si="0"/>
         <v>0.86008230452674894</v>
       </c>
@@ -5259,7 +5336,7 @@
       <c r="C19">
         <v>5</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="5">
         <f t="shared" si="0"/>
         <v>0.97706422018348627</v>
       </c>
@@ -5274,7 +5351,7 @@
       <c r="C20">
         <v>38</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="5">
         <f t="shared" si="0"/>
         <v>0.85098039215686272</v>
       </c>
@@ -5289,7 +5366,7 @@
       <c r="C21">
         <v>40</v>
       </c>
-      <c r="D21" s="9">
+      <c r="D21" s="5">
         <f t="shared" si="0"/>
         <v>0.84674329501915713</v>
       </c>
@@ -5304,7 +5381,7 @@
       <c r="C22">
         <v>112</v>
       </c>
-      <c r="D22" s="9">
+      <c r="D22" s="5">
         <f t="shared" si="0"/>
         <v>0.66765578635014833</v>
       </c>
@@ -5319,7 +5396,7 @@
       <c r="C23">
         <v>44</v>
       </c>
-      <c r="D23" s="9">
+      <c r="D23" s="5">
         <f t="shared" si="0"/>
         <v>0.83882783882783885</v>
       </c>
@@ -5334,7 +5411,7 @@
       <c r="C24">
         <v>46</v>
       </c>
-      <c r="D24" s="9">
+      <c r="D24" s="5">
         <f t="shared" si="0"/>
         <v>0.83512544802867383</v>
       </c>
@@ -5349,7 +5426,7 @@
       <c r="C25">
         <v>4</v>
       </c>
-      <c r="D25" s="9">
+      <c r="D25" s="5">
         <f t="shared" si="0"/>
         <v>0.98340248962655596</v>
       </c>
@@ -5364,7 +5441,7 @@
       <c r="C26">
         <v>50</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="5">
         <f t="shared" si="0"/>
         <v>0.82817869415807566</v>
       </c>
@@ -5379,7 +5456,7 @@
       <c r="C27">
         <v>52</v>
       </c>
-      <c r="D27" s="9">
+      <c r="D27" s="5">
         <f t="shared" si="0"/>
         <v>0.82491582491582494</v>
       </c>
@@ -5394,7 +5471,7 @@
       <c r="C28">
         <v>3</v>
       </c>
-      <c r="D28" s="9">
+      <c r="D28" s="5">
         <f t="shared" si="0"/>
         <v>0.98809523809523814</v>
       </c>
@@ -5409,7 +5486,7 @@
       <c r="C29">
         <v>56</v>
       </c>
-      <c r="D29" s="9">
+      <c r="D29" s="5">
         <f t="shared" si="0"/>
         <v>0.81877022653721687</v>
       </c>
@@ -5424,7 +5501,7 @@
       <c r="C30">
         <v>58</v>
       </c>
-      <c r="D30" s="9">
+      <c r="D30" s="5">
         <f t="shared" si="0"/>
         <v>0.81587301587301586</v>
       </c>
@@ -5439,7 +5516,7 @@
       <c r="C31">
         <v>8</v>
       </c>
-      <c r="D31" s="9">
+      <c r="D31" s="5">
         <f t="shared" si="0"/>
         <v>0.97026022304832715</v>
       </c>
@@ -5454,7 +5531,7 @@
       <c r="C32">
         <v>62</v>
       </c>
-      <c r="D32" s="9">
+      <c r="D32" s="5">
         <f t="shared" si="0"/>
         <v>0.81039755351681952</v>
       </c>
@@ -5469,7 +5546,7 @@
       <c r="C33">
         <v>64</v>
       </c>
-      <c r="D33" s="9">
+      <c r="D33" s="5">
         <f t="shared" si="0"/>
         <v>0.80780780780780781</v>
       </c>
@@ -5484,7 +5561,7 @@
       <c r="C34">
         <v>6</v>
       </c>
-      <c r="D34" s="9">
+      <c r="D34" s="5">
         <f t="shared" si="0"/>
         <v>0.978494623655914</v>
       </c>
@@ -5499,7 +5576,7 @@
       <c r="C35">
         <v>68</v>
       </c>
-      <c r="D35" s="9">
+      <c r="D35" s="5">
         <f t="shared" si="0"/>
         <v>0.80289855072463767</v>
       </c>
@@ -5514,7 +5591,7 @@
       <c r="C36">
         <v>70</v>
       </c>
-      <c r="D36" s="9">
+      <c r="D36" s="5">
         <f t="shared" si="0"/>
         <v>0.80056980056980054</v>
       </c>
@@ -5529,7 +5606,7 @@
       <c r="C37">
         <v>1215</v>
       </c>
-      <c r="D37" s="9">
+      <c r="D37" s="5">
         <f t="shared" si="0"/>
         <v>0.19</v>
       </c>
@@ -5544,7 +5621,7 @@
       <c r="C38">
         <v>74</v>
       </c>
-      <c r="D38" s="9">
+      <c r="D38" s="5">
         <f t="shared" si="0"/>
         <v>0.79614325068870528</v>
       </c>
@@ -5559,7 +5636,7 @@
       <c r="C39">
         <v>76</v>
       </c>
-      <c r="D39" s="9">
+      <c r="D39" s="5">
         <f t="shared" si="0"/>
         <v>0.79403794037940378</v>
       </c>
@@ -5574,7 +5651,7 @@
       <c r="C40">
         <v>5</v>
       </c>
-      <c r="D40" s="9">
+      <c r="D40" s="5">
         <f t="shared" si="0"/>
         <v>0.95798319327731096</v>
       </c>
@@ -5589,7 +5666,7 @@
       <c r="C41">
         <v>0</v>
       </c>
-      <c r="D41" s="9">
+      <c r="D41" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5603,7 +5680,7 @@
       <c r="C42">
         <v>0</v>
       </c>
-      <c r="D42" s="9">
+      <c r="D42" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5617,7 +5694,7 @@
       <c r="C43">
         <v>0</v>
       </c>
-      <c r="D43" s="9">
+      <c r="D43" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5631,7 +5708,7 @@
       <c r="C44">
         <v>0</v>
       </c>
-      <c r="D44" s="9">
+      <c r="D44" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5645,7 +5722,7 @@
       <c r="C45">
         <v>0</v>
       </c>
-      <c r="D45" s="9">
+      <c r="D45" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5659,7 +5736,7 @@
       <c r="C46">
         <v>0</v>
       </c>
-      <c r="D46" s="9">
+      <c r="D46" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5673,7 +5750,7 @@
       <c r="C47">
         <v>0</v>
       </c>
-      <c r="D47" s="9">
+      <c r="D47" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5687,7 +5764,7 @@
       <c r="C48">
         <v>0</v>
       </c>
-      <c r="D48" s="9">
+      <c r="D48" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5701,7 +5778,7 @@
       <c r="C49">
         <v>1</v>
       </c>
-      <c r="D49" s="9">
+      <c r="D49" s="5">
         <f t="shared" ref="D49" si="1">B49/(B49+C49)</f>
         <v>0.98571428571428577</v>
       </c>
@@ -5716,7 +5793,7 @@
       <c r="C50">
         <v>0</v>
       </c>
-      <c r="D50" s="9">
+      <c r="D50" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5730,7 +5807,7 @@
       <c r="C51">
         <v>0</v>
       </c>
-      <c r="D51" s="9">
+      <c r="D51" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5744,7 +5821,7 @@
       <c r="C52">
         <v>0</v>
       </c>
-      <c r="D52" s="9">
+      <c r="D52" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5758,7 +5835,7 @@
       <c r="C53">
         <v>0</v>
       </c>
-      <c r="D53" s="9">
+      <c r="D53" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5772,7 +5849,7 @@
       <c r="C54">
         <v>0</v>
       </c>
-      <c r="D54" s="9">
+      <c r="D54" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5786,7 +5863,7 @@
       <c r="C55">
         <v>0</v>
       </c>
-      <c r="D55" s="9">
+      <c r="D55" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5800,7 +5877,7 @@
       <c r="C56">
         <v>0</v>
       </c>
-      <c r="D56" s="9">
+      <c r="D56" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5814,7 +5891,7 @@
       <c r="C57">
         <v>0</v>
       </c>
-      <c r="D57" s="9">
+      <c r="D57" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5828,7 +5905,7 @@
       <c r="C58">
         <v>0</v>
       </c>
-      <c r="D58" s="9">
+      <c r="D58" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5842,7 +5919,7 @@
       <c r="C59">
         <v>0</v>
       </c>
-      <c r="D59" s="9">
+      <c r="D59" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5856,7 +5933,7 @@
       <c r="C60">
         <v>0</v>
       </c>
-      <c r="D60" s="9">
+      <c r="D60" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5870,7 +5947,7 @@
       <c r="C61">
         <v>0</v>
       </c>
-      <c r="D61" s="9">
+      <c r="D61" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5884,7 +5961,7 @@
       <c r="C62">
         <v>0</v>
       </c>
-      <c r="D62" s="9">
+      <c r="D62" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5898,7 +5975,7 @@
       <c r="C63">
         <v>0</v>
       </c>
-      <c r="D63" s="9">
+      <c r="D63" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5912,7 +5989,7 @@
       <c r="C64">
         <v>0</v>
       </c>
-      <c r="D64" s="9">
+      <c r="D64" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5926,7 +6003,7 @@
       <c r="C65">
         <v>0</v>
       </c>
-      <c r="D65" s="9">
+      <c r="D65" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5940,7 +6017,7 @@
       <c r="C66">
         <v>0</v>
       </c>
-      <c r="D66" s="9">
+      <c r="D66" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5954,7 +6031,7 @@
       <c r="C67">
         <v>0</v>
       </c>
-      <c r="D67" s="9">
+      <c r="D67" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5968,7 +6045,7 @@
       <c r="C68">
         <v>0</v>
       </c>
-      <c r="D68" s="9">
+      <c r="D68" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5982,7 +6059,7 @@
       <c r="C69">
         <v>0</v>
       </c>
-      <c r="D69" s="9">
+      <c r="D69" s="5">
         <v>0</v>
       </c>
     </row>
@@ -5996,7 +6073,7 @@
       <c r="C70">
         <v>0</v>
       </c>
-      <c r="D70" s="9">
+      <c r="D70" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6010,7 +6087,7 @@
       <c r="C71">
         <v>0</v>
       </c>
-      <c r="D71" s="9">
+      <c r="D71" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6024,7 +6101,7 @@
       <c r="C72">
         <v>0</v>
       </c>
-      <c r="D72" s="9">
+      <c r="D72" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6038,7 +6115,7 @@
       <c r="C73">
         <v>0</v>
       </c>
-      <c r="D73" s="9">
+      <c r="D73" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6052,7 +6129,7 @@
       <c r="C74">
         <v>0</v>
       </c>
-      <c r="D74" s="9">
+      <c r="D74" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6066,7 +6143,7 @@
       <c r="C75">
         <v>0</v>
       </c>
-      <c r="D75" s="9">
+      <c r="D75" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6080,7 +6157,7 @@
       <c r="C76">
         <v>0</v>
       </c>
-      <c r="D76" s="9">
+      <c r="D76" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6094,7 +6171,7 @@
       <c r="C77">
         <v>0</v>
       </c>
-      <c r="D77" s="9">
+      <c r="D77" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6108,7 +6185,7 @@
       <c r="C78">
         <v>0</v>
       </c>
-      <c r="D78" s="9">
+      <c r="D78" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6122,7 +6199,7 @@
       <c r="C79">
         <v>0</v>
       </c>
-      <c r="D79" s="9">
+      <c r="D79" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6136,7 +6213,7 @@
       <c r="C80">
         <v>0</v>
       </c>
-      <c r="D80" s="9">
+      <c r="D80" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6150,7 +6227,7 @@
       <c r="C81">
         <v>0</v>
       </c>
-      <c r="D81" s="9">
+      <c r="D81" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6164,7 +6241,7 @@
       <c r="C82">
         <v>0</v>
       </c>
-      <c r="D82" s="9">
+      <c r="D82" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6178,7 +6255,7 @@
       <c r="C83">
         <v>0</v>
       </c>
-      <c r="D83" s="9">
+      <c r="D83" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6192,7 +6269,7 @@
       <c r="C84">
         <v>0</v>
       </c>
-      <c r="D84" s="9">
+      <c r="D84" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6206,7 +6283,7 @@
       <c r="C85">
         <v>0</v>
       </c>
-      <c r="D85" s="9">
+      <c r="D85" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6220,7 +6297,7 @@
       <c r="C86">
         <v>0</v>
       </c>
-      <c r="D86" s="9">
+      <c r="D86" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6234,7 +6311,7 @@
       <c r="C87">
         <v>0</v>
       </c>
-      <c r="D87" s="9">
+      <c r="D87" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6248,7 +6325,7 @@
       <c r="C88">
         <v>0</v>
       </c>
-      <c r="D88" s="9">
+      <c r="D88" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6262,7 +6339,7 @@
       <c r="C89">
         <v>0</v>
       </c>
-      <c r="D89" s="9">
+      <c r="D89" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6276,7 +6353,7 @@
       <c r="C90">
         <v>0</v>
       </c>
-      <c r="D90" s="9">
+      <c r="D90" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6290,7 +6367,7 @@
       <c r="C91">
         <v>0</v>
       </c>
-      <c r="D91" s="9">
+      <c r="D91" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6304,7 +6381,7 @@
       <c r="C92">
         <v>0</v>
       </c>
-      <c r="D92" s="9">
+      <c r="D92" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6318,7 +6395,7 @@
       <c r="C93">
         <v>0</v>
       </c>
-      <c r="D93" s="9">
+      <c r="D93" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6332,7 +6409,7 @@
       <c r="C94">
         <v>15</v>
       </c>
-      <c r="D94" s="9">
+      <c r="D94" s="5">
         <f t="shared" ref="D94" si="2">B94/(B94+C94)</f>
         <v>0.8214285714285714</v>
       </c>
@@ -6347,7 +6424,7 @@
       <c r="C95">
         <v>0</v>
       </c>
-      <c r="D95" s="9">
+      <c r="D95" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6361,7 +6438,7 @@
       <c r="C96">
         <v>0</v>
       </c>
-      <c r="D96" s="9">
+      <c r="D96" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6375,7 +6452,7 @@
       <c r="C97">
         <v>0</v>
       </c>
-      <c r="D97" s="9">
+      <c r="D97" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6389,7 +6466,7 @@
       <c r="C98">
         <v>0</v>
       </c>
-      <c r="D98" s="9">
+      <c r="D98" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6403,7 +6480,7 @@
       <c r="C99">
         <v>0</v>
       </c>
-      <c r="D99" s="9">
+      <c r="D99" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6417,7 +6494,7 @@
       <c r="C100">
         <v>0</v>
       </c>
-      <c r="D100" s="9">
+      <c r="D100" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6431,7 +6508,7 @@
       <c r="C101">
         <v>0</v>
       </c>
-      <c r="D101" s="9">
+      <c r="D101" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6445,7 +6522,7 @@
       <c r="C102">
         <v>0</v>
       </c>
-      <c r="D102" s="9">
+      <c r="D102" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6459,7 +6536,7 @@
       <c r="C103">
         <v>0</v>
       </c>
-      <c r="D103" s="9">
+      <c r="D103" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6473,7 +6550,7 @@
       <c r="C104">
         <v>0</v>
       </c>
-      <c r="D104" s="9">
+      <c r="D104" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6487,7 +6564,7 @@
       <c r="C105">
         <v>0</v>
       </c>
-      <c r="D105" s="9">
+      <c r="D105" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6501,7 +6578,7 @@
       <c r="C106">
         <v>0</v>
       </c>
-      <c r="D106" s="9">
+      <c r="D106" s="5">
         <v>0</v>
       </c>
     </row>
@@ -6515,7 +6592,7 @@
       <c r="C107">
         <v>0</v>
       </c>
-      <c r="D107" s="9">
+      <c r="D107" s="5">
         <v>0</v>
       </c>
     </row>

</xml_diff>